<commit_message>
GL-4 DD_LISA_P1 small update to match P2
</commit_message>
<xml_diff>
--- a/rmonize/data_dictionary/DD_LISA_P1.xlsx
+++ b/rmonize/data_dictionary/DD_LISA_P1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20415"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Projekte\NFDI4Health\TA5\Pilotprojekte\Harmonisierung\HarmonizR\use-cases-harmonisation\rmonize\data_dictionary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{30B8857A-D1A5-43D7-9D93-F1F7668B42E8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BE44F3B-8BED-40B1-A352-D418CC600C5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{1200B70D-B446-4CDA-99A8-3FD394D791D2}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11025" windowHeight="11760" activeTab="1" xr2:uid="{1200B70D-B446-4CDA-99A8-3FD394D791D2}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -26,10 +26,10 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="214">
   <si>
     <t>index</t>
   </si>
@@ -639,27 +639,6 @@
     <t>female</t>
   </si>
   <si>
-    <t>No secondary school or elementary school certificate (Mother)</t>
-  </si>
-  <si>
-    <t>Lower secondary school or elementary school certificate (Mother)</t>
-  </si>
-  <si>
-    <t>Secondary school certificate (middle school leaving certificate)(Mother)</t>
-  </si>
-  <si>
-    <t>Completion of Polytechnic. high school (Mother)</t>
-  </si>
-  <si>
-    <t>Advanced technical college entrance qualification (Mother)</t>
-  </si>
-  <si>
-    <t>General or specialist university entrance qualification (Mother)</t>
-  </si>
-  <si>
-    <t>Other degree (Mother)</t>
-  </si>
-  <si>
     <t>No secondary school or elementary school certificate</t>
   </si>
   <si>
@@ -694,6 +673,12 @@
   </si>
   <si>
     <t>yes, less often</t>
+  </si>
+  <si>
+    <t>Other degree</t>
+  </si>
+  <si>
+    <t>General or specialist university entrance qualification</t>
   </si>
 </sst>
 </file>
@@ -804,7 +789,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -820,9 +805,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -860,7 +845,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -966,7 +951,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1108,7 +1093,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1117,7 +1102,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08A73012-5CAD-43B9-A281-79101DF4E1E0}">
   <dimension ref="A1:D96"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="3"/>
     <col min="2" max="2" width="26.28515625" style="5" customWidth="1"/>
@@ -2478,7 +2463,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7CFBFAA-22DC-428C-A718-7E0BADD40216}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.42578125" style="3"/>
@@ -2519,7 +2504,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>12</v>
       </c>
@@ -2530,7 +2515,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>12</v>
       </c>
@@ -2582,7 +2567,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -2593,7 +2578,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2604,7 +2589,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2615,7 +2600,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -2626,7 +2611,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2637,7 +2622,7 @@
         <v>4</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2648,7 +2633,7 @@
         <v>5</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2659,7 +2644,7 @@
         <v>6</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2670,7 +2655,7 @@
         <v>7</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -2681,7 +2666,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -2692,7 +2677,7 @@
         <v>2</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -2703,7 +2688,7 @@
         <v>3</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2714,7 +2699,7 @@
         <v>4</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -2725,7 +2710,7 @@
         <v>5</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -2734,15 +2719,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
@@ -2752,6 +2728,15 @@
     <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2996,14 +2981,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C05FF1B-7508-40EF-8319-E993EA07F007}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D9CBEFE-8C4C-4054-8E02-CA457E93B4C8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -3016,6 +2993,14 @@
     <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C05FF1B-7508-40EF-8319-E993EA07F007}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>